<commit_message>
Change logging from text file to Excel file with trailing SL support
- Updated log_order_placement() to use Excel logging instead of text file
- Added Excel logging for all trade events (entry, exit, trailing SL updates)
- Fixed import path for excel_logger using sys.path.insert
- Added TYPE_CHECKING to excel_logger for proper type hints
- Enhanced trailing SL implementation with Excel logging:
  * Logs trailing SL updates with old/new SL and profit
  * Logs SL_HIT, TRAILED_SL_HIT, and TARGET_HIT events
  * Each event includes entry, current price, P&L
- All trade data now logged to signal_logs.xlsx with two sheets:
  * Signal Checks: Entry signal detection logs
  * Trades: Order placement, exits, and trailing SL updates
- Fixed syntax errors in excel_logger.py with TYPE_CHECKING pattern
</commit_message>
<xml_diff>
--- a/Mine/signal_logs.xlsx
+++ b/Mine/signal_logs.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -987,6 +987,132 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 10:45:00</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>10:45:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 10:50:00</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>10:50:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 10:55:00</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>10:55:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix 5-minute interval logging to prevent missing entries after hour boundaries
- Added last_entry_check_time tracking to ensure each 5-minute interval checked exactly once
- Updated should_check_entry_signal() to track interval completion vs time window
- Replaced narrow 10-second window with interval-based tracking
- Added Excel logging for EVERY 5-minute check regardless of signal status
- Logs now include 'NO' for no signals and 'YES' for signals with full details
- Fixed missing logs at 14:00, 14:05, 14:10, 14:15 after 13:55
- Added failed data fetch logging to Excel for troubleshooting
- Updated reset_daily() to reset last_entry_check_time

Now logs all 5-minute intervals: 9:15, 9:20, 9:25... 14:00, 14:05... 15:20
without missing any checks due to processing delays or hour boundaries.
</commit_message>
<xml_diff>
--- a/Mine/signal_logs.xlsx
+++ b/Mine/signal_logs.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1113,6 +1113,1392 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 11:20:00</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>11:20:00</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 11:25:00</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>11:25:00</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 11:30:00</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>11:30:00</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 11:35:00</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>11:35:00</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 11:40:00</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>11:40:00</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 11:47:39</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>11:47:39</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>11:47</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 11:50:00</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>11:50:00</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 11:55:00</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>11:55:00</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:20:00</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>12:20:00</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:26:58</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>12:26:58</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>12:26</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:30:00</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:35:00</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>12:35:00</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:40:00</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>12:40:00</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:45:00</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>12:45:00</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:50:00</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>12:50:00</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:55:00</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>12:55:00</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 13:20:38</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>13:20:38</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 13:25:00</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>13:25:00</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 13:30:00</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>13:30:00</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 13:35:00</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>13:35:00</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 13:40:00</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 13:45:00</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 13:50:00</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 13:55:00</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 14:20:00</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 14:25:00</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>14:25:00</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 14:30:00</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>14:30:00</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 14:35:00</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>14:35:00</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 14:40:00</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>14:40:00</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 14:45:00</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 14:50:00</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 14:55:00</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>14:55:00</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 15:20:38</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>15:20:38</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr"/>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>